<commit_message>
Add PDFs for refs 01-06, remove duplicate, link all papers in tracking sheets
</commit_message>
<xml_diff>
--- a/FYP - Saad Mazhar/02 Literature/Paper Tracking Matrix.xlsx
+++ b/FYP - Saad Mazhar/02 Literature/Paper Tracking Matrix.xlsx
@@ -565,14 +565,13 @@
       </c>
       <c r="O2" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIR is referred to as a "green" tool because it reduces the need for the chemical reagents typically used in laboratory tea analysis
-. The principle of NIR is explained through the analogy of looking into a room: while "specular reflectance" only shows the shape of a window, "diffuse reflectance" allows the sensor to see the objects (chemical components) inside the sample
-</t>
-        </is>
-      </c>
-      <c r="P2" s="11" t="inlineStr">
-        <is>
-          <t>PDF not uploaded yet</t>
+          <t>NIR is referred to as a "green" tool because it reduces the need for the chemical reagents typically used in laboratory tea analysis
+. The principle of NIR is explained through the analogy of looking into a room: while "specular reflectance" only shows the shape of a window, "diffuse reflectance" allows the sensor to see the objects (chemical components) inside the sample Stored PDF is a 1-page scan from Two and a Bud.</t>
+        </is>
+      </c>
+      <c r="P2" s="12" t="inlineStr">
+        <is>
+          <t>01 - Hazarika 2017 - Near Infrared (NIR) Spectroscopy - The green analytical tool for tea quality analyses.pdf</t>
         </is>
       </c>
     </row>
@@ -613,7 +612,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>ANS2020 (The document notes this was an Oral Presentation)</t>
+          <t>1st Asian NIR Symposium (ANS2020) - oral presentation abstract</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -678,9 +677,9 @@
           <t>A key finding of the paper was the significant improvement in data quality through processing; the Separability Index (SI) increased from 53.63 for the raw dataset to 93.20 after applying pre-processing techniques"</t>
         </is>
       </c>
-      <c r="P4" s="11" t="inlineStr">
-        <is>
-          <t>PDF not uploaded yet</t>
+      <c r="P4" s="12" t="inlineStr">
+        <is>
+          <t>02 - Das 2020 - Discrimination of Green Tea Samples on the Basis of Gallic Acid Content Using Near Infrared Spectroscopy.pdf</t>
         </is>
       </c>
     </row>
@@ -798,9 +797,9 @@
 </t>
         </is>
       </c>
-      <c r="P6" s="11" t="inlineStr">
-        <is>
-          <t>PDF not uploaded yet</t>
+      <c r="P6" s="12" t="inlineStr">
+        <is>
+          <t>03 - Revilla 2024 - The Potential Use of Near Infrared Spectroscopy (NIRS) to Determine Heavy Metals and Blend Percentage in Tea.pdf</t>
         </is>
       </c>
     </row>
@@ -841,7 +840,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Not explicitly mentioned in the text (the source filename suggests a submission for a conference in Rome)</t>
+          <t>Conference abstract (filename indicates a Rome conference, 2024; event name not printed in the PDF)</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -906,9 +905,9 @@
           <t>The CARS-PLSR model provided the best performance for TF, liquor, and quality (with an Rp of 0.983 for TF), while the RF-PLSR model was more effective for predicting infusion scores</t>
         </is>
       </c>
-      <c r="P8" s="11" t="inlineStr">
-        <is>
-          <t>PDF not uploaded yet</t>
+      <c r="P8" s="12" t="inlineStr">
+        <is>
+          <t>04 - Hazarika 2024 - Rapid Quality Evaluation and Market Valuation of CTC Black Tea Using Near Infrared Spectroscopy.pdf</t>
         </is>
       </c>
     </row>
@@ -1034,9 +1033,9 @@
 Some misidentifications occurred in comprehensive tests due to non-uniform roasting</t>
         </is>
       </c>
-      <c r="P10" s="11" t="inlineStr">
-        <is>
-          <t>PDF not uploaded yet</t>
+      <c r="P10" s="12" t="inlineStr">
+        <is>
+          <t>05 - Huang 2024 - Terahertz Spectroscopic Identification of Roast Degree and Variety of Coffee Beans.pdf</t>
         </is>
       </c>
     </row>
@@ -1143,9 +1142,9 @@
 . Additionally, it notes that Raman spectroscopy is uniquely valuable because it is insensitive to moisture, unlike many other infrared techniques</t>
         </is>
       </c>
-      <c r="P12" s="11" t="inlineStr">
-        <is>
-          <t>PDF not uploaded yet</t>
+      <c r="P12" s="12" t="inlineStr">
+        <is>
+          <t>06 - Qiu 2026 - Research progress of spectroscopic detection technology in agricultural product quality detection.pdf</t>
         </is>
       </c>
     </row>
@@ -4346,59 +4345,65 @@
   <autoFilter ref="A1:P104"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P50" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P52" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P60" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P64" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P66" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P68" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P32" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P34" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P36" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P38" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P40" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P46" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P48" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P50" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P52" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P54" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P56" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P58" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P60" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P62" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P64" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P66" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P68" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>